<commit_message>
Fix clipped Suggestion-block cells: set explicit row height for wrapped text
Excel never auto-fits row height across a merged cell, only unmerged
ones - since every Suggestion cell is a merge spanning the plant's
original row span, a multi-line wrapped value (the bulleted Remark
worst of all) stayed at the template's original short row height and
got visually clipped at the bottom, most visibly on the last row.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MG2nzeeWa5SnWqcTDjXsda
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__merge_mode_gpt4omini.xlsx
+++ b/pfmea_ai/NEW_PFMEA__merge_mode_gpt4omini.xlsx
@@ -2408,7 +2408,7 @@
       <c r="AS17" s="208" t="n"/>
       <c r="AT17" s="208" t="n"/>
     </row>
-    <row r="18" ht="102" customFormat="1" customHeight="1" s="8">
+    <row r="18" ht="142.5" customFormat="1" customHeight="1" s="8">
       <c r="A18" s="120" t="inlineStr">
         <is>
           <t>HEAD LAMP STAGE</t>
@@ -3318,7 +3318,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="118.5" customFormat="1" customHeight="1" s="13">
+    <row r="29" ht="240" customFormat="1" customHeight="1" s="13">
       <c r="B29" s="210" t="n"/>
       <c r="C29" s="211" t="n"/>
       <c r="D29" s="210" t="n"/>

</xml_diff>

<commit_message>
Split reviewer flag into dedicated AI Review + Manual Review columns
Remark stays LLM-automated-only (merged mode, cause/mismatch, ambiguity,
plant-vs-AI disagreement, duplicate cause) instead of getting overloaded
with human-facing findings. New columns:
  AI Review     - deeper cross-check findings (e.g. the row 5 Effect-list
                  gap), separate from the per-row LLM output
  Manual Review - left blank for the plant engineer's own decision

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MG2nzeeWa5SnWqcTDjXsda
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__merge_mode_gpt4omini.xlsx
+++ b/pfmea_ai/NEW_PFMEA__merge_mode_gpt4omini.xlsx
@@ -1611,7 +1611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT29"/>
+  <dimension ref="A1:AV29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.85546875" customWidth="1" min="1" max="1"/>
@@ -1624,6 +1624,8 @@
     <col width="40" customWidth="1" min="44" max="44"/>
     <col width="45" customWidth="1" min="45" max="45"/>
     <col width="50" customWidth="1" min="46" max="46"/>
+    <col width="45" customWidth="1" min="47" max="47"/>
+    <col width="35" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customFormat="1" customHeight="1" s="1">
@@ -2066,6 +2068,8 @@
       <c r="AR13" s="205" t="n"/>
       <c r="AS13" s="205" t="n"/>
       <c r="AT13" s="205" t="n"/>
+      <c r="AU13" s="205" t="n"/>
+      <c r="AV13" s="205" t="n"/>
     </row>
     <row r="14" ht="22.5" customFormat="1" customHeight="1" s="1">
       <c r="A14" s="198" t="n"/>
@@ -2114,6 +2118,8 @@
       <c r="AR14" s="205" t="n"/>
       <c r="AS14" s="205" t="n"/>
       <c r="AT14" s="205" t="n"/>
+      <c r="AU14" s="205" t="n"/>
+      <c r="AV14" s="205" t="n"/>
     </row>
     <row r="15" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A15" s="91" t="inlineStr">
@@ -2309,6 +2315,16 @@
       <c r="AT15" s="208" t="inlineStr">
         <is>
           <t>Remark</t>
+        </is>
+      </c>
+      <c r="AU15" s="208" t="inlineStr">
+        <is>
+          <t>AI Review</t>
+        </is>
+      </c>
+      <c r="AV15" s="208" t="inlineStr">
+        <is>
+          <t>Manual Review</t>
         </is>
       </c>
     </row>
@@ -2359,6 +2375,8 @@
       <c r="AR16" s="208" t="n"/>
       <c r="AS16" s="208" t="n"/>
       <c r="AT16" s="208" t="n"/>
+      <c r="AU16" s="208" t="n"/>
+      <c r="AV16" s="208" t="n"/>
     </row>
     <row r="17" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A17" s="198" t="n"/>
@@ -2407,6 +2425,8 @@
       <c r="AR17" s="208" t="n"/>
       <c r="AS17" s="208" t="n"/>
       <c r="AT17" s="208" t="n"/>
+      <c r="AU17" s="208" t="n"/>
+      <c r="AV17" s="208" t="n"/>
     </row>
     <row r="18" ht="142.5" customFormat="1" customHeight="1" s="8">
       <c r="A18" s="120" t="inlineStr">
@@ -2575,6 +2595,8 @@
 ( NOT AS PER MODEL). Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
+      <c r="AU18" s="223" t="inlineStr"/>
+      <c r="AV18" s="223" t="inlineStr"/>
     </row>
     <row r="19" ht="207" customFormat="1" customHeight="1" s="8">
       <c r="B19" s="210" t="n"/>
@@ -2627,6 +2649,8 @@
       <c r="AR19" s="223" t="n"/>
       <c r="AS19" s="223" t="n"/>
       <c r="AT19" s="223" t="n"/>
+      <c r="AU19" s="223" t="n"/>
+      <c r="AV19" s="223" t="n"/>
     </row>
     <row r="20" ht="117" customFormat="1" customHeight="1" s="8">
       <c r="B20" s="210" t="n"/>
@@ -2713,6 +2737,8 @@
 - Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
+      <c r="AU20" s="223" t="inlineStr"/>
+      <c r="AV20" s="223" t="inlineStr"/>
     </row>
     <row r="21" ht="153" customFormat="1" customHeight="1" s="8">
       <c r="B21" s="210" t="n"/>
@@ -2765,6 +2791,8 @@
       <c r="AR21" s="223" t="n"/>
       <c r="AS21" s="223" t="n"/>
       <c r="AT21" s="223" t="n"/>
+      <c r="AU21" s="223" t="n"/>
+      <c r="AV21" s="223" t="n"/>
     </row>
     <row r="22" ht="119.25" customFormat="1" customHeight="1" s="8">
       <c r="B22" s="210" t="n"/>
@@ -2855,6 +2883,8 @@
           <t>- AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
       </c>
+      <c r="AU22" s="223" t="inlineStr"/>
+      <c r="AV22" s="223" t="inlineStr"/>
     </row>
     <row r="23" ht="186.95" customFormat="1" customHeight="1" s="14">
       <c r="B23" s="210" t="n"/>
@@ -2927,6 +2957,8 @@
       <c r="AR23" s="223" t="n"/>
       <c r="AS23" s="223" t="n"/>
       <c r="AT23" s="223" t="n"/>
+      <c r="AU23" s="223" t="n"/>
+      <c r="AV23" s="223" t="n"/>
     </row>
     <row r="24" ht="130.5" customFormat="1" customHeight="1" s="14">
       <c r="B24" s="210" t="n"/>
@@ -3006,6 +3038,8 @@
           <t>- AI severity (10) differs from plant-recorded (5) - review recommended.</t>
         </is>
       </c>
+      <c r="AU24" s="223" t="inlineStr"/>
+      <c r="AV24" s="223" t="inlineStr"/>
     </row>
     <row r="25" ht="130.5" customFormat="1" customHeight="1" s="14">
       <c r="B25" s="210" t="n"/>
@@ -3062,6 +3096,8 @@
       <c r="AR25" s="223" t="n"/>
       <c r="AS25" s="223" t="n"/>
       <c r="AT25" s="223" t="n"/>
+      <c r="AU25" s="223" t="n"/>
+      <c r="AV25" s="223" t="n"/>
     </row>
     <row r="26" ht="135" customFormat="1" customHeight="1" s="14">
       <c r="B26" s="210" t="n"/>
@@ -3163,6 +3199,8 @@
           <t>- Merged failure mode (2 distinct modes detected) - see the A/B breakdown in Severity/Detection/Prevention above, matched against the Failure Mode text.</t>
         </is>
       </c>
+      <c r="AU26" s="223" t="inlineStr"/>
+      <c r="AV26" s="223" t="inlineStr"/>
     </row>
     <row r="27" ht="156" customFormat="1" customHeight="1" s="13">
       <c r="B27" s="210" t="n"/>
@@ -3225,6 +3263,8 @@
       <c r="AR27" s="223" t="n"/>
       <c r="AS27" s="223" t="n"/>
       <c r="AT27" s="223" t="n"/>
+      <c r="AU27" s="223" t="n"/>
+      <c r="AV27" s="223" t="n"/>
     </row>
     <row r="28" ht="151.5" customFormat="1" customHeight="1" s="13">
       <c r="B28" s="210" t="n"/>
@@ -3317,6 +3357,8 @@
           <t>- Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED - OVER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
+      <c r="AU28" s="223" t="inlineStr"/>
+      <c r="AV28" s="223" t="inlineStr"/>
     </row>
     <row r="29" ht="240" customFormat="1" customHeight="1" s="13">
       <c r="B29" s="210" t="n"/>
@@ -3399,10 +3441,12 @@
 - Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
+      <c r="AU29" s="223" t="inlineStr"/>
+      <c r="AV29" s="223" t="inlineStr"/>
     </row>
     <row r="30" customFormat="1" s="18"/>
   </sheetData>
-  <mergeCells count="169">
+  <mergeCells count="181">
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="K18:L29"/>
     <mergeCell ref="I24:J25"/>
@@ -3410,6 +3454,7 @@
     <mergeCell ref="AM15:AM17"/>
     <mergeCell ref="AT18:AT19"/>
     <mergeCell ref="AE15:AE17"/>
+    <mergeCell ref="AV18:AV19"/>
     <mergeCell ref="AG15:AG17"/>
     <mergeCell ref="C15:D17"/>
     <mergeCell ref="K10:T10"/>
@@ -3420,18 +3465,20 @@
     <mergeCell ref="T13:AA14"/>
     <mergeCell ref="S1:T2"/>
     <mergeCell ref="D12:F12"/>
+    <mergeCell ref="AU24:AU25"/>
     <mergeCell ref="D9:F9"/>
     <mergeCell ref="G13:L14"/>
     <mergeCell ref="AR24:AR25"/>
     <mergeCell ref="K9:T9"/>
     <mergeCell ref="K5:T5"/>
     <mergeCell ref="T28:U29"/>
+    <mergeCell ref="AU26:AU27"/>
     <mergeCell ref="AN15:AN17"/>
     <mergeCell ref="AT26:AT27"/>
     <mergeCell ref="K11:T11"/>
     <mergeCell ref="I3:T4"/>
     <mergeCell ref="AS18:AS19"/>
-    <mergeCell ref="AM13:AT14"/>
+    <mergeCell ref="AU18:AU19"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="AM22:AM23"/>
     <mergeCell ref="K12:T12"/>
@@ -3451,7 +3498,9 @@
     <mergeCell ref="AQ20:AQ21"/>
     <mergeCell ref="T15:U17"/>
     <mergeCell ref="AN24:AN25"/>
+    <mergeCell ref="AM13:AV14"/>
     <mergeCell ref="AT15:AT17"/>
+    <mergeCell ref="AV15:AV17"/>
     <mergeCell ref="K7:T7"/>
     <mergeCell ref="R19:S19"/>
     <mergeCell ref="A12:C12"/>
@@ -3485,6 +3534,7 @@
     <mergeCell ref="AC15:AC17"/>
     <mergeCell ref="R28:S29"/>
     <mergeCell ref="I26:J27"/>
+    <mergeCell ref="AV20:AV21"/>
     <mergeCell ref="AQ24:AQ25"/>
     <mergeCell ref="AS24:AS25"/>
     <mergeCell ref="AD15:AD17"/>
@@ -3496,6 +3546,8 @@
     <mergeCell ref="I28:J29"/>
     <mergeCell ref="AF15:AF17"/>
     <mergeCell ref="AS20:AS21"/>
+    <mergeCell ref="AU20:AU21"/>
+    <mergeCell ref="AV22:AV23"/>
     <mergeCell ref="AQ26:AQ27"/>
     <mergeCell ref="AS26:AS27"/>
     <mergeCell ref="P15:Q17"/>
@@ -3517,13 +3569,16 @@
     <mergeCell ref="AM20:AM21"/>
     <mergeCell ref="W28:X29"/>
     <mergeCell ref="P20:Q21"/>
+    <mergeCell ref="AV24:AV25"/>
     <mergeCell ref="R22:S22"/>
     <mergeCell ref="AO22:AO23"/>
     <mergeCell ref="P22:Q23"/>
     <mergeCell ref="AR22:AR23"/>
     <mergeCell ref="V18:V21"/>
     <mergeCell ref="AT22:AT23"/>
+    <mergeCell ref="AV26:AV27"/>
     <mergeCell ref="T19:U19"/>
+    <mergeCell ref="AU15:AU17"/>
     <mergeCell ref="AO15:AO17"/>
     <mergeCell ref="D6:F6"/>
     <mergeCell ref="V27:V29"/>
@@ -3569,6 +3624,7 @@
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="T23:U23"/>
     <mergeCell ref="D10:F10"/>
+    <mergeCell ref="AU22:AU23"/>
     <mergeCell ref="AR26:AR27"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="T18:U18"/>

</xml_diff>

<commit_message>
Fix lost red/bold formatting on plant's own rich-text cells
load_workbook() without rich_text=True silently flattens a cell's
per-run formatting (e.g. the bold/red 'Your Plant :' / 'Ship to Plant :'
/ 'End User :' labels inside Failure Effect) into one plain string on
load, so re-saving dropped that inline styling even though this script
never touches those cells' content. Passing rich_text=True preserves it.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MG2nzeeWa5SnWqcTDjXsda
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__merge_mode_gpt4omini.xlsx
+++ b/pfmea_ai/NEW_PFMEA__merge_mode_gpt4omini.xlsx
@@ -2124,9 +2124,31 @@
     <row r="15" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A15" s="91" t="inlineStr">
         <is>
-          <t>1. Process Item System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>System, Subsystem,
 Part Element or
 Name of Process</t>
+          </r>
         </is>
       </c>
       <c r="B15" s="207" t="n"/>
@@ -2145,8 +2167,30 @@
       <c r="F15" s="207" t="n"/>
       <c r="G15" s="102" t="inlineStr">
         <is>
-          <t>1. Function of the Process Item Function of System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Function of the Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>Function of System, Subsystem,
 Part Element or Process</t>
+          </r>
         </is>
       </c>
       <c r="H15" s="207" t="n"/>
@@ -2437,36 +2481,293 @@
       <c r="B18" s="207" t="n"/>
       <c r="C18" s="218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operation No: 
-Stage: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Operation No</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Stage:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> 
 RH / LH HEAD LAMP FITMENT
 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
         </is>
       </c>
       <c r="D18" s="207" t="n"/>
       <c r="E18" s="219" t="inlineStr">
         <is>
-          <t>1 Man - Operator
-2.Machine-  
+          <r>
+            <t xml:space="preserve">1 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Man </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- Operator
+2.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Machine</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-  
 Battery tool, Traceability scanner
-3.Material (Indirect) - PPE's
-4.Method-
+3.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Material (Indirect)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> - PPE's
+4.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Method</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-
 Connections, Bolt fitment
-5.Mother Nature
-(Environment)-NA
-6.Measurement- NA</t>
+5.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Mother Nature
+(Environment)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-NA
+6.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Measurement</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- NA</t>
+          </r>
         </is>
       </c>
       <c r="F18" s="207" t="n"/>
       <c r="G18" s="220" t="inlineStr">
         <is>
-          <t>Your Plant :
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 Headlamp assembly in specific design (bulb/LED assembly, lens fitting, aiming, electrical connection)
-Ship to Plant : 
-End User : 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">End User </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Provide adequate illumination of the road ahead during low-light or night conditions
 2. Ensure visibility of the vehicle to other road users
 3. Meet legal/regulatory lighting requirements (beam pattern, intensity, color)</t>
+          </r>
         </is>
       </c>
       <c r="H18" s="207" t="n"/>
@@ -2478,32 +2779,185 @@
       <c r="J18" s="207" t="n"/>
       <c r="K18" s="221" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Man: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Man: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. COLLECT THE HEAD LAMP LH / RH SIDE FROM STORAGE AREA AND SCAN THE PART
 2. CONNECT THE 2 CONNECTORS WITH HEAD LAMP
 3. ALIGN THE HEAD LAMP WITH THE BIW AND THEN TIGHT WITH BOLTS
-2. Machine:
-Proper torquing with 6NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">2. Machine:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Proper torquing with 6NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 3. Material (Indirect) :
-Hand Gloves, Apron
-4. Method:
-1. Install Head lamp from sequencing trolley and scan
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Hand Gloves, Apron
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">4. Method:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Install Head lamp from sequencing trolley and scan
 2. Align H/L with BIW, then do the connections with wiring harness with head lamp and tight with bolts
 </t>
+          </r>
         </is>
       </c>
       <c r="L18" s="207" t="n"/>
       <c r="M18" s="161" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Wrong Head lamp variant installed
 2. FURTHER OPERATION NOT POSSIBLE
 3. Lens cracked or broken
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Headlamp does not turn ON
 2. Insufficient brightness / dim light
 3. Customer dissatisfaction</t>
+          </r>
         </is>
       </c>
       <c r="N18" s="207" t="n"/>
@@ -2812,16 +3266,82 @@
       <c r="L22" s="210" t="n"/>
       <c r="M22" s="224" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Wiring harness partially connected (loose fitment)
 2. Electrical connector loose or damaged
 3. Rework time required high and further fitment not possible 
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Incorrect beam alignment
 2. Headlamp does not turn ON
 3. Reduced road visibility
 4. Increased risk of accident</t>
+          </r>
         </is>
       </c>
       <c r="N22" s="207" t="n"/>
@@ -3117,16 +3637,103 @@
       <c r="L26" s="210" t="n"/>
       <c r="M26" s="224" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. DAMAGE OF THREADS / RATTLING DUE TO JOINT LOOSE
 2. Mounting screws under-torqued or over-torqued
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Lens cracked or broken
 2. LED / BULB burnout
 3. Water ingress inside lamp
 4. Rattling or vibration noise during driving
 5. Driver discomfort or eye strain</t>
+          </r>
         </is>
       </c>
       <c r="N26" s="207" t="n"/>
@@ -4120,9 +4727,31 @@
     <row r="15" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A15" s="91" t="inlineStr">
         <is>
-          <t>1. Process Item System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>System, Subsystem,
 Part Element or
 Name of Process</t>
+          </r>
         </is>
       </c>
       <c r="B15" s="207" t="n"/>
@@ -4141,8 +4770,30 @@
       <c r="F15" s="207" t="n"/>
       <c r="G15" s="102" t="inlineStr">
         <is>
-          <t>1. Function of the Process Item Function of System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Function of the Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>Function of System, Subsystem,
 Part Element or Process</t>
+          </r>
         </is>
       </c>
       <c r="H15" s="207" t="n"/>
@@ -4363,37 +5014,294 @@
       <c r="B18" s="207" t="n"/>
       <c r="C18" s="218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operation No: 
-Stage: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Operation No</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Stage:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> 
 FRONT GRILL FITMENT- HIGH VARIANT
 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
         </is>
       </c>
       <c r="D18" s="207" t="n"/>
       <c r="E18" s="219" t="inlineStr">
         <is>
-          <t>1 Man - Operator
-2.Machine-  
+          <r>
+            <t xml:space="preserve">1 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Man </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- Operator
+2.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Machine</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-  
 Battery tool, Traceability scanner
-3.Material (Indirect) - PPE's
-4.Method-
+3.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Material (Indirect)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> - PPE's
+4.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Method</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-
 Connections, 
 Bolts &amp; pushpin   fitment
-5.Mother Nature
-(Environment)-NA
-6.Measurement- NA</t>
+5.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Mother Nature
+(Environment)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-NA
+6.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Measurement</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- NA</t>
+          </r>
         </is>
       </c>
       <c r="F18" s="207" t="n"/>
       <c r="G18" s="220" t="inlineStr">
         <is>
-          <t>Your Plant :
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 To correctly install front grill fitment as per BIW design specifications.
-Ship to Plant : 
-End User : 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">End User </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Allow airflow to the radiator, condenser, and engine compartment
 2. Protect cooling components from debris, stones, insects
 3. Provide vehicle styling and brand identity</t>
+          </r>
         </is>
       </c>
       <c r="H18" s="207" t="n"/>
@@ -4405,33 +5313,186 @@
       <c r="J18" s="207" t="n"/>
       <c r="K18" s="221" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Man: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Man: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. TAKE THE FRONT GRILL FROM THE STORAGE AREA AND SCAN THE PART
 2. CONNECT THE CONNECTORS WITH GRILL
 3. INSERT &amp; 
 ALIGN THE FRONT GRILL WITH BIW AND THEN TIGHT WITH BOLTS AND PUSHPINS
-2. Machine:
-Proper torquing with 4NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">2. Machine:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Proper torquing with 4NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 3. Material (Indirect) :
-Hand Gloves, Apron
-4. Method:
-1. Install Front grill from sequencing trolley and scan
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Hand Gloves, Apron
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">4. Method:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Install Front grill from sequencing trolley and scan
 2. Then do the connections with wiring harness with grill and align with BIW and tight with bolts &amp; pushpins
 </t>
+          </r>
         </is>
       </c>
       <c r="L18" s="207" t="n"/>
       <c r="M18" s="161" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Wrong front grill variant installed
 2. FURTHER OPERATION NOT POSSIBLE
 3. Gaps or scratches on grill 
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Incorrect distance / object detection
 2. Water/dust ingress affecting sensor
 3. Customer dissatisfaction</t>
+          </r>
         </is>
       </c>
       <c r="N18" s="207" t="n"/>
@@ -4629,16 +5690,82 @@
       <c r="L22" s="210" t="n"/>
       <c r="M22" s="224" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Wiring harness partially connected (loose fitment)
 2. Wiring harness pinched or damaged
 3. Rework time required high and further fitment not possible 
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. False ADAS warnings or alerts
 2. Incorrect object detection
 3. Lane assist / collision warning inoperative
 4. Increased risk of accident</t>
+          </r>
         </is>
       </c>
       <c r="N22" s="207" t="n"/>
@@ -4845,16 +5972,103 @@
       <c r="L26" s="210" t="n"/>
       <c r="M26" s="224" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. DAMAGE OF THREADS / RATTLING DUE TO JOINT LOOSE
 2. Mounting bolts under-torqued or over-torqued
 3. Broken clips
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Customer loss of confidence in vehicle safety
 2. False collision warnings provided to driver
 3. Water/dust ingress affecting sensor
 4. Rattling or vibration noise during driving</t>
+          </r>
         </is>
       </c>
       <c r="N26" s="207" t="n"/>
@@ -5656,9 +6870,31 @@
     <row r="15" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A15" s="91" t="inlineStr">
         <is>
-          <t>1. Process Item System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>System, Subsystem,
 Part Element or
 Name of Process</t>
+          </r>
         </is>
       </c>
       <c r="B15" s="207" t="n"/>
@@ -5677,8 +6913,30 @@
       <c r="F15" s="207" t="n"/>
       <c r="G15" s="102" t="inlineStr">
         <is>
-          <t>1. Function of the Process Item Function of System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Function of the Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>Function of System, Subsystem,
 Part Element or Process</t>
+          </r>
         </is>
       </c>
       <c r="H15" s="207" t="n"/>
@@ -5899,36 +7157,293 @@
       <c r="B18" s="207" t="n"/>
       <c r="C18" s="218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operation No: 
-Stage: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Operation No</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Stage:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> 
 FRONT GRILL FITMENT- LOW VARIANT
 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
         </is>
       </c>
       <c r="D18" s="207" t="n"/>
       <c r="E18" s="219" t="inlineStr">
         <is>
-          <t>1 Man - Operator
-2.Machine-  
+          <r>
+            <t xml:space="preserve">1 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Man </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- Operator
+2.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Machine</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-  
 Battery tool, Traceability scanner
-3.Material (Indirect) - PPE's
-4.Method-
+3.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Material (Indirect)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> - PPE's
+4.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Method</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-
 Bolts &amp; pushpin   fitment
-5.Mother Nature
-(Environment)-NA
-6.Measurement- NA</t>
+5.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Mother Nature
+(Environment)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-NA
+6.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Measurement</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- NA</t>
+          </r>
         </is>
       </c>
       <c r="F18" s="207" t="n"/>
       <c r="G18" s="220" t="inlineStr">
         <is>
-          <t>Your Plant :
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 To correctly install front grill fitment as per BIW design specifications.
-Ship to Plant : 
-End User : 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">End User </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Allow airflow to the radiator, condenser, and engine compartment
 2. Protect cooling components from debris, stones, insects
 3. Provide vehicle styling and brand identity</t>
+          </r>
         </is>
       </c>
       <c r="H18" s="207" t="n"/>
@@ -5940,32 +7455,185 @@
       <c r="J18" s="207" t="n"/>
       <c r="K18" s="221" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Man: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Man: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. TAKE THE FRONT GRILL FROM THE STORAGE AREA AND SCAN THE PART
 2. INSERT &amp; 
 ALIGN THE FRONT GRILL WITH BIW AND THEN TIGHT WITH BOLTS AND PUSHPINS
-2. Machine:
-Proper torquing with 4NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">2. Machine:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Proper torquing with 4NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 3. Material (Indirect) :
-Hand Gloves, Apron
-4. Method:
-1. Install Front grill from sequencing trolley and scan
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Hand Gloves, Apron
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">4. Method:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Install Front grill from sequencing trolley and scan
 2. Align with BIW and tight with bolts &amp; pushpins
 </t>
+          </r>
         </is>
       </c>
       <c r="L18" s="207" t="n"/>
       <c r="M18" s="161" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Wrong front grill variant installed
 2. FURTHER OPERATION NOT POSSIBLE
 3. Gaps or scratches on grill 
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Water/dust ingress affecting sensor
 2. Customer dissatisfaction
 3. Bad appereance of vehicle</t>
+          </r>
         </is>
       </c>
       <c r="N18" s="207" t="n"/>
@@ -6126,11 +7794,77 @@
       <c r="L21" s="210" t="n"/>
       <c r="M21" s="161" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Rework time required high and further fitment not possible 
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Water/dust ingress affecting part warrenty</t>
+          </r>
         </is>
       </c>
       <c r="N21" s="207" t="n"/>
@@ -6306,14 +8040,101 @@
       <c r="L24" s="210" t="n"/>
       <c r="M24" s="224" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. DAMAGE OF THREADS / RATTLING DUE TO JOINT LOOSE
 2. Mounting bolts under-torqued or over-torqued
 3. Broken clips
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Water/dust ingress affecting sensor
 2. Rattling or vibration noise during driving</t>
+          </r>
         </is>
       </c>
       <c r="N24" s="207" t="n"/>
@@ -7127,9 +8948,31 @@
     <row r="15" ht="22.5" customFormat="1" customHeight="1" s="6">
       <c r="A15" s="91" t="inlineStr">
         <is>
-          <t>1. Process Item System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>System, Subsystem,
 Part Element or
 Name of Process</t>
+          </r>
         </is>
       </c>
       <c r="B15" s="207" t="n"/>
@@ -7148,8 +8991,30 @@
       <c r="F15" s="207" t="n"/>
       <c r="G15" s="102" t="inlineStr">
         <is>
-          <t>1. Function of the Process Item Function of System, Subsystem,
+          <r>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">Function of the Process Item </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>Function of System, Subsystem,
 Part Element or Process</t>
+          </r>
         </is>
       </c>
       <c r="H15" s="207" t="n"/>
@@ -7370,37 +9235,294 @@
       <c r="B18" s="207" t="n"/>
       <c r="C18" s="218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operation No: 
-Stage: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Operation No</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Stage:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> 
 LH / RH RADIATOR SIDE SEAL FITMENT
 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
         </is>
       </c>
       <c r="D18" s="207" t="n"/>
       <c r="E18" s="219" t="inlineStr">
         <is>
-          <t>1 Man - Operator
-2.Machine-  
+          <r>
+            <t xml:space="preserve">1 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Man </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- Operator
+2.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Machine</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-  
 Battery tool
-3.Material (Indirect) - PPE's
-4.Method-
+3.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Material (Indirect)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> - PPE's
+4.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Method</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-
 Screw &amp; pushpin fitment
-5.Mother Nature
-(Environment)-NA
-6.Measurement- NA</t>
+5.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Mother Nature
+(Environment)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>-NA
+6.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Measurement</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>- NA</t>
+          </r>
         </is>
       </c>
       <c r="F18" s="207" t="n"/>
       <c r="G18" s="220" t="inlineStr">
         <is>
-          <t>Your Plant :
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Correct installation and positioning of the side seal during radiator assembly.
 2. Maintain seal integrity (no cuts, twists or misalignment)
-Ship to Plant : 
-End User : 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">End User </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Maintain system pressure under operating temperature and vibration
 2. Accommodate thermal expansion between radiator components
 3. Seal the joint between the radiator core and side tank to prevent coolant leakage</t>
+          </r>
         </is>
       </c>
       <c r="H18" s="207" t="n"/>
@@ -7412,30 +9534,183 @@
       <c r="J18" s="207" t="n"/>
       <c r="K18" s="221" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Man: 
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Man: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. GET THE SIDE SEAL FROM STORAGE BIN
 2. ALIGN THE SIDE SEAL WITH THE BIW AND THEN TIGHT WITH BOLT AND PUSHPIN
-2. Machine:
-Proper torquing with 6NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">2. Machine:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Proper torquing with 6NM
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 3. Material (Indirect) :
-Hand Gloves, Apron
-4. Method:
-1. Take side seal from storage bin
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Hand Gloves, Apron
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">4. Method:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">1. Take side seal from storage bin
 2. Align side seal with BIW and tight with bolt and pushpin
 </t>
+          </r>
         </is>
       </c>
       <c r="L18" s="207" t="n"/>
       <c r="M18" s="161" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Wrong part installed or mixed material
 2. FURTHER OPERATION NOT POSSIBLE
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Vehicle overheating
 2. Coolant seepage or visible leak
 3. Customer dissatisfaction</t>
+          </r>
         </is>
       </c>
       <c r="N18" s="207" t="n"/>
@@ -7544,15 +9819,81 @@
       <c r="L20" s="210" t="n"/>
       <c r="M20" s="224" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Cut, torn, pinched, or cracked seal
 2. Seal under-compressed or over-compressed
 3. Rework time required high and further fitment not possible 
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">Ship to Plant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Reduced cooling efficiency
 2. Engine overheating
 3. Safety risk if overheating occurs during driving</t>
+          </r>
         </is>
       </c>
       <c r="N20" s="207" t="n"/>
@@ -7821,14 +10162,101 @@
       <c r="L25" s="210" t="n"/>
       <c r="M25" s="161" t="inlineStr">
         <is>
-          <t>Your Plant:
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Your Plant:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. DAMAGE OF THREADS / RATTLING DUE TO JOINT LOOSE
 2. Mounting Bolt under-torqued or over-torqued
-Ship to Plant : Nil
-End User:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Ship to Plant :</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Nil</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>End User:</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 1. Customer dissatisfaction due to coolant leak
 2. Coolant dripping under vehicle
 3. Rattling or vibration noise during driving</t>
+          </r>
         </is>
       </c>
       <c r="N25" s="207" t="n"/>

</xml_diff>